<commit_message>
Fix login button and admin navigation performance
- Rewrite login page as server component with native form action (no JS
  hydration dependency — button works even before React loads)
- Add adminLoginFormAction that handles cookie + redirect server-side
- Replace force-dynamic with revalidate=30 on all admin pages so pages
  are served from edge cache instead of cold-starting on every click
- Add revalidatePath calls to all mutating actions so cache is
  invalidated immediately after any data change
- Fix JWT secret read at module-load time (function-level instead)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/modelo-convidados.xlsx
+++ b/public/modelo-convidados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJETOS\Zoe1\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{522BDF46-2D2B-498E-AB56-248D10435FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57F9A93B-ACCD-4877-9C36-0668C58042F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="26">
   <si>
     <t>Responsável</t>
   </si>
@@ -480,7 +480,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.875" customWidth="1"/>
     <col min="2" max="2" width="16.875" customWidth="1"/>
@@ -497,7 +497,7 @@
     <col min="13" max="13" width="10.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,7 +538,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -567,7 +567,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -590,7 +590,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -613,13 +613,19 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>25</v>
       </c>
       <c r="B5">
         <v>21994329471</v>
       </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>13</v>
+      </c>
       <c r="H5" t="s">
         <v>15</v>
       </c>
@@ -639,7 +645,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="H6" t="s">
         <v>15</v>
       </c>

</xml_diff>